<commit_message>
chore(examples): regenerate playoffs example workbooks for bracket-order numbering
cmd/create-playoffs.go now numbers competitors after StandardSeeding
(bc-pnum ruling 2), so any example roster with a dojo collision
delayDojoMeetings had to repair changes numbering order. Only the
four examples with an actual reorder to make changed:
playoffs-example-large(-seeded).xlsx and
playoffs-example-medium(-seeded).xlsx. playoffs-example-small.xlsx
and every pools-example-*.xlsx are confirmed byte-identical to before
(verified via sha256 against the pre-change commit) -- create-pools.go
and the small fixture's roster have nothing for delayDojoMeetings to
move, so numbering before or after seeding gives the same order there.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/playoffs-example-medium-seeded.xlsx
+++ b/playoffs-example-medium-seeded.xlsx
@@ -92,6 +92,177 @@
     <t>K1</t>
   </si>
   <si>
+    <t>Gandalf The Grey</t>
+  </si>
+  <si>
+    <t>Team Eta</t>
+  </si>
+  <si>
+    <t>GANDALF</t>
+  </si>
+  <si>
+    <t>K2</t>
+  </si>
+  <si>
+    <t>Hermione Granger</t>
+  </si>
+  <si>
+    <t>Team Theta</t>
+  </si>
+  <si>
+    <t>GRANGER</t>
+  </si>
+  <si>
+    <t>K3</t>
+  </si>
+  <si>
+    <t>Inigo Montoya</t>
+  </si>
+  <si>
+    <t>Team Iota</t>
+  </si>
+  <si>
+    <t>MONTOYA</t>
+  </si>
+  <si>
+    <t>K4</t>
+  </si>
+  <si>
+    <t>Jon Snow</t>
+  </si>
+  <si>
+    <t>Team Kappa</t>
+  </si>
+  <si>
+    <t>SNOW</t>
+  </si>
+  <si>
+    <t>K5</t>
+  </si>
+  <si>
+    <t>Katniss Everdeen</t>
+  </si>
+  <si>
+    <t>Team Lambda</t>
+  </si>
+  <si>
+    <t>EVERDEEN</t>
+  </si>
+  <si>
+    <t>K6</t>
+  </si>
+  <si>
+    <t>Petyr Baelish</t>
+  </si>
+  <si>
+    <t>Team Pi</t>
+  </si>
+  <si>
+    <t>BAELISH</t>
+  </si>
+  <si>
+    <t>K7</t>
+  </si>
+  <si>
+    <t>Legolas Greenleaf</t>
+  </si>
+  <si>
+    <t>Team Mu</t>
+  </si>
+  <si>
+    <t>GREENLEAF</t>
+  </si>
+  <si>
+    <t>K8</t>
+  </si>
+  <si>
+    <t>Frodo Baggins</t>
+  </si>
+  <si>
+    <t>Team Zeta</t>
+  </si>
+  <si>
+    <t>BAGGINS</t>
+  </si>
+  <si>
+    <t>K9</t>
+  </si>
+  <si>
+    <t>Moby Dick</t>
+  </si>
+  <si>
+    <t>Team Nu</t>
+  </si>
+  <si>
+    <t>DICK</t>
+  </si>
+  <si>
+    <t>K10</t>
+  </si>
+  <si>
+    <t>Neville Longbottom</t>
+  </si>
+  <si>
+    <t>Team Xi</t>
+  </si>
+  <si>
+    <t>LONGBOTTOM</t>
+  </si>
+  <si>
+    <t>K11</t>
+  </si>
+  <si>
+    <t>Othello</t>
+  </si>
+  <si>
+    <t>Team Omicron</t>
+  </si>
+  <si>
+    <t>OTHELLO</t>
+  </si>
+  <si>
+    <t>K12</t>
+  </si>
+  <si>
+    <t>K13</t>
+  </si>
+  <si>
+    <t>Quirinus Quirrell</t>
+  </si>
+  <si>
+    <t>Team Rho</t>
+  </si>
+  <si>
+    <t>QUIRRELL</t>
+  </si>
+  <si>
+    <t>K14</t>
+  </si>
+  <si>
+    <t>Ron Weasley</t>
+  </si>
+  <si>
+    <t>Team Sigma</t>
+  </si>
+  <si>
+    <t>WEASLEY</t>
+  </si>
+  <si>
+    <t>K15</t>
+  </si>
+  <si>
+    <t>Samwise Gamgee</t>
+  </si>
+  <si>
+    <t>Team Tau</t>
+  </si>
+  <si>
+    <t>GAMGEE</t>
+  </si>
+  <si>
+    <t>K16</t>
+  </si>
+  <si>
     <t>Daenerys Targaryen</t>
   </si>
   <si>
@@ -101,7 +272,76 @@
     <t>TARGARYEN</t>
   </si>
   <si>
-    <t>K2</t>
+    <t>K17</t>
+  </si>
+  <si>
+    <t>Tyrion Lannister</t>
+  </si>
+  <si>
+    <t>Team Upsilon</t>
+  </si>
+  <si>
+    <t>K18</t>
+  </si>
+  <si>
+    <t>Ulysses</t>
+  </si>
+  <si>
+    <t>Team Phi</t>
+  </si>
+  <si>
+    <t>ULYSSES</t>
+  </si>
+  <si>
+    <t>K19</t>
+  </si>
+  <si>
+    <t>Voldemort</t>
+  </si>
+  <si>
+    <t>Team Chi</t>
+  </si>
+  <si>
+    <t>VOLDEMORT</t>
+  </si>
+  <si>
+    <t>K20</t>
+  </si>
+  <si>
+    <t>Willy Wonka</t>
+  </si>
+  <si>
+    <t>Team Psi</t>
+  </si>
+  <si>
+    <t>WONKA</t>
+  </si>
+  <si>
+    <t>K21</t>
+  </si>
+  <si>
+    <t>Xaro Xhoan Daxos</t>
+  </si>
+  <si>
+    <t>Team Omega</t>
+  </si>
+  <si>
+    <t>DAXOS</t>
+  </si>
+  <si>
+    <t>K22</t>
+  </si>
+  <si>
+    <t>Ygritte</t>
+  </si>
+  <si>
+    <t>Team Alpha</t>
+  </si>
+  <si>
+    <t>YGRITTE</t>
+  </si>
+  <si>
+    <t>K23</t>
   </si>
   <si>
     <t>Eddard Stark</t>
@@ -111,246 +351,6 @@
   </si>
   <si>
     <t>STARK</t>
-  </si>
-  <si>
-    <t>K3</t>
-  </si>
-  <si>
-    <t>Frodo Baggins</t>
-  </si>
-  <si>
-    <t>Team Zeta</t>
-  </si>
-  <si>
-    <t>BAGGINS</t>
-  </si>
-  <si>
-    <t>K4</t>
-  </si>
-  <si>
-    <t>Gandalf The Grey</t>
-  </si>
-  <si>
-    <t>Team Eta</t>
-  </si>
-  <si>
-    <t>GANDALF</t>
-  </si>
-  <si>
-    <t>K5</t>
-  </si>
-  <si>
-    <t>Hermione Granger</t>
-  </si>
-  <si>
-    <t>Team Theta</t>
-  </si>
-  <si>
-    <t>GRANGER</t>
-  </si>
-  <si>
-    <t>K6</t>
-  </si>
-  <si>
-    <t>Inigo Montoya</t>
-  </si>
-  <si>
-    <t>Team Iota</t>
-  </si>
-  <si>
-    <t>MONTOYA</t>
-  </si>
-  <si>
-    <t>K7</t>
-  </si>
-  <si>
-    <t>Jon Snow</t>
-  </si>
-  <si>
-    <t>Team Kappa</t>
-  </si>
-  <si>
-    <t>SNOW</t>
-  </si>
-  <si>
-    <t>K8</t>
-  </si>
-  <si>
-    <t>Katniss Everdeen</t>
-  </si>
-  <si>
-    <t>Team Lambda</t>
-  </si>
-  <si>
-    <t>EVERDEEN</t>
-  </si>
-  <si>
-    <t>K9</t>
-  </si>
-  <si>
-    <t>Team Mu</t>
-  </si>
-  <si>
-    <t>K10</t>
-  </si>
-  <si>
-    <t>Legolas Greenleaf</t>
-  </si>
-  <si>
-    <t>GREENLEAF</t>
-  </si>
-  <si>
-    <t>K11</t>
-  </si>
-  <si>
-    <t>Moby Dick</t>
-  </si>
-  <si>
-    <t>Team Nu</t>
-  </si>
-  <si>
-    <t>DICK</t>
-  </si>
-  <si>
-    <t>K12</t>
-  </si>
-  <si>
-    <t>Neville Longbottom</t>
-  </si>
-  <si>
-    <t>Team Xi</t>
-  </si>
-  <si>
-    <t>LONGBOTTOM</t>
-  </si>
-  <si>
-    <t>K13</t>
-  </si>
-  <si>
-    <t>Othello</t>
-  </si>
-  <si>
-    <t>Team Omicron</t>
-  </si>
-  <si>
-    <t>OTHELLO</t>
-  </si>
-  <si>
-    <t>K14</t>
-  </si>
-  <si>
-    <t>Petyr Baelish</t>
-  </si>
-  <si>
-    <t>Team Pi</t>
-  </si>
-  <si>
-    <t>BAELISH</t>
-  </si>
-  <si>
-    <t>K15</t>
-  </si>
-  <si>
-    <t>Quirinus Quirrell</t>
-  </si>
-  <si>
-    <t>Team Rho</t>
-  </si>
-  <si>
-    <t>QUIRRELL</t>
-  </si>
-  <si>
-    <t>K16</t>
-  </si>
-  <si>
-    <t>Ron Weasley</t>
-  </si>
-  <si>
-    <t>Team Sigma</t>
-  </si>
-  <si>
-    <t>WEASLEY</t>
-  </si>
-  <si>
-    <t>K17</t>
-  </si>
-  <si>
-    <t>Samwise Gamgee</t>
-  </si>
-  <si>
-    <t>Team Tau</t>
-  </si>
-  <si>
-    <t>GAMGEE</t>
-  </si>
-  <si>
-    <t>K18</t>
-  </si>
-  <si>
-    <t>Tyrion Lannister</t>
-  </si>
-  <si>
-    <t>Team Upsilon</t>
-  </si>
-  <si>
-    <t>K19</t>
-  </si>
-  <si>
-    <t>Ulysses</t>
-  </si>
-  <si>
-    <t>Team Phi</t>
-  </si>
-  <si>
-    <t>ULYSSES</t>
-  </si>
-  <si>
-    <t>K20</t>
-  </si>
-  <si>
-    <t>Voldemort</t>
-  </si>
-  <si>
-    <t>Team Chi</t>
-  </si>
-  <si>
-    <t>VOLDEMORT</t>
-  </si>
-  <si>
-    <t>K21</t>
-  </si>
-  <si>
-    <t>Willy Wonka</t>
-  </si>
-  <si>
-    <t>Team Psi</t>
-  </si>
-  <si>
-    <t>WONKA</t>
-  </si>
-  <si>
-    <t>K22</t>
-  </si>
-  <si>
-    <t>Xaro Xhoan Daxos</t>
-  </si>
-  <si>
-    <t>Team Omega</t>
-  </si>
-  <si>
-    <t>DAXOS</t>
-  </si>
-  <si>
-    <t>K23</t>
-  </si>
-  <si>
-    <t>Ygritte</t>
-  </si>
-  <si>
-    <t>Team Alpha</t>
-  </si>
-  <si>
-    <t>YGRITTE</t>
   </si>
   <si>
     <t>K24</t>
@@ -1045,7 +1045,7 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>21</v>
@@ -1062,7 +1062,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
         <v>25</v>
@@ -1079,7 +1079,7 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>29</v>
@@ -1096,7 +1096,7 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
         <v>33</v>
@@ -1113,7 +1113,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
         <v>37</v>
@@ -1130,7 +1130,7 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
         <v>41</v>
@@ -1147,7 +1147,7 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
         <v>45</v>
@@ -1164,7 +1164,7 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B11" t="s">
         <v>49</v>
@@ -1181,67 +1181,67 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E13" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C14" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E14" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="D15" t="s">
-        <v>64</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
         <v>65</v>
@@ -1249,7 +1249,7 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
         <v>66</v>
@@ -1266,7 +1266,7 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
         <v>70</v>
@@ -1283,7 +1283,7 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B18" t="s">
         <v>74</v>
@@ -1300,7 +1300,7 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="B19" t="s">
         <v>78</v>
@@ -1317,7 +1317,7 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
         <v>82</v>
@@ -1326,24 +1326,24 @@
         <v>83</v>
       </c>
       <c r="D20" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20" t="s">
         <v>84</v>
-      </c>
-      <c r="E20" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" t="s">
         <v>86</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>87</v>
-      </c>
-      <c r="D21" t="s">
-        <v>19</v>
       </c>
       <c r="E21" t="s">
         <v>88</v>
@@ -1351,7 +1351,7 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
         <v>89</v>
@@ -1368,7 +1368,7 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>93</v>
@@ -1385,7 +1385,7 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24" t="s">
         <v>97</v>
@@ -1402,7 +1402,7 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25" t="s">
         <v>101</v>
@@ -1419,7 +1419,7 @@
     </row>
     <row r="26">
       <c r="A26">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="B26" t="s">
         <v>105</v>
@@ -1458,90 +1458,90 @@
     </row>
     <row r="2" ht="270" customHeight="true">
       <c r="A2" s="17" t="str">
-        <f>'data'!$E$7</f>
+        <f>'data'!$E$4</f>
       </c>
       <c r="B2" s="18" t="str">
-        <f>'data'!D7</f>
+        <f>'data'!D4</f>
       </c>
     </row>
     <row r="3" ht="270" customHeight="true">
       <c r="A3" s="17" t="str">
-        <f>'data'!$E$8</f>
+        <f>'data'!$E$5</f>
       </c>
       <c r="B3" s="18" t="str">
-        <f>'data'!D8</f>
+        <f>'data'!D5</f>
       </c>
     </row>
     <row r="4" ht="270" customHeight="true">
       <c r="A4" s="17" t="str">
-        <f>'data'!$E$9</f>
+        <f>'data'!$E$6</f>
       </c>
       <c r="B4" s="18" t="str">
-        <f>'data'!D9</f>
+        <f>'data'!D6</f>
       </c>
     </row>
     <row r="5" ht="270" customHeight="true">
       <c r="A5" s="17" t="str">
-        <f>'data'!$E$10</f>
+        <f>'data'!$E$7</f>
       </c>
       <c r="B5" s="18" t="str">
-        <f>'data'!D10</f>
+        <f>'data'!D7</f>
       </c>
     </row>
     <row r="6" ht="270" customHeight="true">
       <c r="A6" s="17" t="str">
-        <f>'data'!$E$11</f>
+        <f>'data'!$E$8</f>
       </c>
       <c r="B6" s="18" t="str">
-        <f>'data'!D11</f>
+        <f>'data'!D8</f>
       </c>
     </row>
     <row r="7" ht="270" customHeight="true">
       <c r="A7" s="17" t="str">
-        <f>'data'!$E$17</f>
+        <f>'data'!$E$9</f>
       </c>
       <c r="B7" s="18" t="str">
-        <f>'data'!D17</f>
+        <f>'data'!D9</f>
       </c>
     </row>
     <row r="8" ht="270" customHeight="true">
       <c r="A8" s="17" t="str">
-        <f>'data'!$E$13</f>
+        <f>'data'!$E$10</f>
       </c>
       <c r="B8" s="18" t="str">
-        <f>'data'!D13</f>
+        <f>'data'!D10</f>
       </c>
     </row>
     <row r="9" ht="270" customHeight="true">
       <c r="A9" s="17" t="str">
-        <f>'data'!$E$6</f>
+        <f>'data'!$E$11</f>
       </c>
       <c r="B9" s="18" t="str">
-        <f>'data'!D6</f>
+        <f>'data'!D11</f>
       </c>
     </row>
     <row r="10" ht="270" customHeight="true">
       <c r="A10" s="17" t="str">
-        <f>'data'!$E$14</f>
+        <f>'data'!$E$12</f>
       </c>
       <c r="B10" s="18" t="str">
-        <f>'data'!D14</f>
+        <f>'data'!D12</f>
       </c>
     </row>
     <row r="11" ht="270" customHeight="true">
       <c r="A11" s="17" t="str">
-        <f>'data'!$E$15</f>
+        <f>'data'!$E$13</f>
       </c>
       <c r="B11" s="18" t="str">
-        <f>'data'!D15</f>
+        <f>'data'!D13</f>
       </c>
     </row>
     <row r="12" ht="270" customHeight="true">
       <c r="A12" s="17" t="str">
-        <f>'data'!$E$16</f>
+        <f>'data'!$E$14</f>
       </c>
       <c r="B12" s="18" t="str">
-        <f>'data'!D16</f>
+        <f>'data'!D14</f>
       </c>
     </row>
   </sheetData>
@@ -1568,98 +1568,98 @@
   <sheetData>
     <row r="1" ht="270" customHeight="true">
       <c r="A1" s="17" t="str">
-        <f>'data'!$E$12</f>
+        <f>'data'!$E$15</f>
       </c>
       <c r="B1" s="18" t="str">
-        <f>'data'!D12</f>
+        <f>'data'!D15</f>
       </c>
     </row>
     <row r="2" ht="270" customHeight="true">
       <c r="A2" s="17" t="str">
-        <f>'data'!$E$18</f>
+        <f>'data'!$E$16</f>
       </c>
       <c r="B2" s="18" t="str">
-        <f>'data'!D18</f>
+        <f>'data'!D16</f>
       </c>
     </row>
     <row r="3" ht="270" customHeight="true">
       <c r="A3" s="17" t="str">
-        <f>'data'!$E$19</f>
+        <f>'data'!$E$17</f>
       </c>
       <c r="B3" s="18" t="str">
-        <f>'data'!D19</f>
+        <f>'data'!D17</f>
       </c>
     </row>
     <row r="4" ht="270" customHeight="true">
       <c r="A4" s="17" t="str">
-        <f>'data'!$E$20</f>
+        <f>'data'!$E$18</f>
       </c>
       <c r="B4" s="18" t="str">
-        <f>'data'!D20</f>
+        <f>'data'!D18</f>
       </c>
     </row>
     <row r="5" ht="270" customHeight="true">
       <c r="A5" s="17" t="str">
-        <f>'data'!$E$4</f>
+        <f>'data'!$E$19</f>
       </c>
       <c r="B5" s="18" t="str">
-        <f>'data'!D4</f>
+        <f>'data'!D19</f>
       </c>
     </row>
     <row r="6" ht="270" customHeight="true">
       <c r="A6" s="17" t="str">
-        <f>'data'!$E$21</f>
+        <f>'data'!$E$20</f>
       </c>
       <c r="B6" s="18" t="str">
-        <f>'data'!D21</f>
+        <f>'data'!D20</f>
       </c>
     </row>
     <row r="7" ht="270" customHeight="true">
       <c r="A7" s="17" t="str">
-        <f>'data'!$E$22</f>
+        <f>'data'!$E$21</f>
       </c>
       <c r="B7" s="18" t="str">
-        <f>'data'!D22</f>
+        <f>'data'!D21</f>
       </c>
     </row>
     <row r="8" ht="270" customHeight="true">
       <c r="A8" s="17" t="str">
-        <f>'data'!$E$23</f>
+        <f>'data'!$E$22</f>
       </c>
       <c r="B8" s="18" t="str">
-        <f>'data'!D23</f>
+        <f>'data'!D22</f>
       </c>
     </row>
     <row r="9" ht="270" customHeight="true">
       <c r="A9" s="17" t="str">
-        <f>'data'!$E$24</f>
+        <f>'data'!$E$23</f>
       </c>
       <c r="B9" s="18" t="str">
-        <f>'data'!D24</f>
+        <f>'data'!D23</f>
       </c>
     </row>
     <row r="10" ht="270" customHeight="true">
       <c r="A10" s="17" t="str">
-        <f>'data'!$E$25</f>
+        <f>'data'!$E$24</f>
       </c>
       <c r="B10" s="18" t="str">
-        <f>'data'!D25</f>
+        <f>'data'!D24</f>
       </c>
     </row>
     <row r="11" ht="270" customHeight="true">
       <c r="A11" s="17" t="str">
-        <f>'data'!$E$26</f>
+        <f>'data'!$E$25</f>
       </c>
       <c r="B11" s="18" t="str">
-        <f>'data'!D26</f>
+        <f>'data'!D25</f>
       </c>
     </row>
     <row r="12" ht="270" customHeight="true">
       <c r="A12" s="17" t="str">
-        <f>'data'!$E$5</f>
+        <f>'data'!$E$26</f>
       </c>
       <c r="B12" s="18" t="str">
-        <f>'data'!D5</f>
+        <f>'data'!D26</f>
       </c>
     </row>
   </sheetData>
@@ -2033,7 +2033,7 @@
     </row>
     <row r="4">
       <c r="A4" s="19" t="str">
-        <f>'data'!$B$8</f>
+        <f>'data'!$B$5</f>
       </c>
       <c r="B4" s="22"/>
       <c r="C4" s="22"/>
@@ -2041,10 +2041,10 @@
       <c r="E4" s="22"/>
       <c r="F4" s="22"/>
       <c r="G4" s="19" t="str">
-        <f>'data'!$B$7</f>
+        <f>'data'!$B$4</f>
       </c>
       <c r="I4" s="19" t="str">
-        <f>'data'!$B$19</f>
+        <f>'data'!$B$17</f>
       </c>
       <c r="J4" s="22"/>
       <c r="K4" s="22"/>
@@ -2052,7 +2052,7 @@
       <c r="M4" s="22"/>
       <c r="N4" s="22"/>
       <c r="O4" s="19" t="str">
-        <f>'data'!$B$18</f>
+        <f>'data'!$B$16</f>
       </c>
     </row>
     <row r="6">
@@ -2117,7 +2117,7 @@
     </row>
     <row r="12">
       <c r="A12" s="19" t="str">
-        <f>'data'!$B$12</f>
+        <f>'data'!$B$15</f>
       </c>
       <c r="B12" s="22"/>
       <c r="C12" s="22"/>
@@ -2125,10 +2125,10 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
       <c r="G12" s="19" t="str">
-        <f>'data'!$B$10</f>
+        <f>'data'!$B$7</f>
       </c>
       <c r="I12" s="19" t="str">
-        <f>'data'!$B$21</f>
+        <f>'data'!$B$20</f>
       </c>
       <c r="J12" s="22"/>
       <c r="K12" s="22"/>
@@ -2136,7 +2136,7 @@
       <c r="M12" s="22"/>
       <c r="N12" s="22"/>
       <c r="O12" s="19" t="str">
-        <f>'data'!$B$4</f>
+        <f>'data'!$B$19</f>
       </c>
     </row>
     <row r="14">
@@ -2201,7 +2201,7 @@
     </row>
     <row r="20">
       <c r="A20" s="19" t="str">
-        <f>'data'!$B$6</f>
+        <f>'data'!$B$11</f>
       </c>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -2209,10 +2209,10 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
       <c r="G20" s="19" t="str">
-        <f>'data'!$B$13</f>
+        <f>'data'!$B$10</f>
       </c>
       <c r="I20" s="19" t="str">
-        <f>'data'!$B$24</f>
+        <f>'data'!$B$23</f>
       </c>
       <c r="J20" s="22"/>
       <c r="K20" s="22"/>
@@ -2220,7 +2220,7 @@
       <c r="M20" s="22"/>
       <c r="N20" s="22"/>
       <c r="O20" s="19" t="str">
-        <f>'data'!$B$23</f>
+        <f>'data'!$B$22</f>
       </c>
     </row>
     <row r="22">
@@ -2285,7 +2285,7 @@
     </row>
     <row r="28">
       <c r="A28" s="19" t="str">
-        <f>'data'!$B$16</f>
+        <f>'data'!$B$14</f>
       </c>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -2293,10 +2293,10 @@
       <c r="E28" s="22"/>
       <c r="F28" s="22"/>
       <c r="G28" s="19" t="str">
-        <f>'data'!$B$15</f>
+        <f>'data'!$B$13</f>
       </c>
       <c r="I28" s="19" t="str">
-        <f>'data'!$B$5</f>
+        <f>'data'!$B$26</f>
       </c>
       <c r="J28" s="22"/>
       <c r="K28" s="22"/>
@@ -2304,7 +2304,7 @@
       <c r="M28" s="22"/>
       <c r="N28" s="22"/>
       <c r="O28" s="19" t="str">
-        <f>'data'!$B$26</f>
+        <f>'data'!$B$25</f>
       </c>
     </row>
     <row r="30">
@@ -2377,7 +2377,7 @@
       <c r="E41" s="22"/>
       <c r="F41" s="22"/>
       <c r="G41" s="19" t="str">
-        <f>'data'!$B$21</f>
+        <f>'data'!$B$20</f>
       </c>
       <c r="I41" s="19" t="str">
         <f>CONCATENATE("M 5 ",O6)</f>
@@ -2388,7 +2388,7 @@
       <c r="M41" s="22"/>
       <c r="N41" s="22"/>
       <c r="O41" s="19" t="str">
-        <f>'data'!$B$12</f>
+        <f>'data'!$B$15</f>
       </c>
     </row>
     <row r="43">
@@ -2461,7 +2461,7 @@
       <c r="E49" s="22"/>
       <c r="F49" s="22"/>
       <c r="G49" s="19" t="str">
-        <f>'data'!$B$9</f>
+        <f>'data'!$B$6</f>
       </c>
       <c r="I49" s="19" t="str">
         <f>CONCATENATE("M 6 ",O14)</f>
@@ -2472,7 +2472,7 @@
       <c r="M49" s="22"/>
       <c r="N49" s="22"/>
       <c r="O49" s="19" t="str">
-        <f>'data'!$B$20</f>
+        <f>'data'!$B$18</f>
       </c>
     </row>
     <row r="51">
@@ -2545,7 +2545,7 @@
       <c r="E57" s="22"/>
       <c r="F57" s="22"/>
       <c r="G57" s="19" t="str">
-        <f>'data'!$B$17</f>
+        <f>'data'!$B$9</f>
       </c>
       <c r="I57" s="19" t="str">
         <f>CONCATENATE("M 7 ",O22)</f>
@@ -2556,7 +2556,7 @@
       <c r="M57" s="22"/>
       <c r="N57" s="22"/>
       <c r="O57" s="19" t="str">
-        <f>'data'!$B$22</f>
+        <f>'data'!$B$21</f>
       </c>
     </row>
     <row r="59">
@@ -2629,7 +2629,7 @@
       <c r="E65" s="22"/>
       <c r="F65" s="22"/>
       <c r="G65" s="19" t="str">
-        <f>'data'!$B$14</f>
+        <f>'data'!$B$12</f>
       </c>
       <c r="I65" s="19" t="str">
         <f>CONCATENATE("M 8 ",O30)</f>
@@ -2640,7 +2640,7 @@
       <c r="M65" s="22"/>
       <c r="N65" s="22"/>
       <c r="O65" s="19" t="str">
-        <f>'data'!$B$25</f>
+        <f>'data'!$B$24</f>
       </c>
     </row>
     <row r="67">
@@ -3050,7 +3050,7 @@
     </row>
     <row r="9">
       <c r="C9" s="16" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="G9" s="12"/>
       <c r="H9" s="14"/>
@@ -3067,7 +3067,7 @@
     </row>
     <row r="11">
       <c r="C11" s="16" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="12"/>
@@ -3087,7 +3087,7 @@
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="I14" s="12"/>
       <c r="K14" s="12"/>
@@ -3108,7 +3108,7 @@
     </row>
     <row r="17">
       <c r="C17" s="16" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="G17" s="12"/>
       <c r="K17" s="12"/>
@@ -3124,7 +3124,7 @@
     </row>
     <row r="19">
       <c r="C19" s="16" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="12"/>
@@ -3142,7 +3142,7 @@
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
       <c r="E22" s="16" t="s">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="K22" s="12"/>
     </row>
@@ -3159,7 +3159,7 @@
     </row>
     <row r="25">
       <c r="C25" s="16" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="14"/>
@@ -3178,7 +3178,7 @@
     </row>
     <row r="27">
       <c r="C27" s="16" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="12"/>
@@ -3199,7 +3199,7 @@
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="I30" s="12"/>
     </row>
@@ -3217,7 +3217,7 @@
     </row>
     <row r="33">
       <c r="C33" s="16" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="G33" s="12"/>
     </row>
@@ -3231,7 +3231,7 @@
     </row>
     <row r="35">
       <c r="C35" s="16" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="12"/>
@@ -3279,7 +3279,7 @@
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
@@ -3293,7 +3293,7 @@
     </row>
     <row r="9">
       <c r="C9" s="16" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G9" s="12"/>
       <c r="H9" s="14"/>
@@ -3310,7 +3310,7 @@
     </row>
     <row r="11">
       <c r="C11" s="16" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="D11" s="15"/>
       <c r="E11" s="12"/>
@@ -3330,7 +3330,7 @@
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="I14" s="12"/>
       <c r="K14" s="12"/>
@@ -3351,7 +3351,7 @@
     </row>
     <row r="17">
       <c r="C17" s="16" t="s">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="G17" s="12"/>
       <c r="K17" s="12"/>
@@ -3385,7 +3385,7 @@
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
       <c r="E22" s="16" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="K22" s="12"/>
     </row>
@@ -3402,7 +3402,7 @@
     </row>
     <row r="25">
       <c r="C25" s="16" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="14"/>
@@ -3421,7 +3421,7 @@
     </row>
     <row r="27">
       <c r="C27" s="16" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="12"/>
@@ -3442,7 +3442,7 @@
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="I30" s="12"/>
     </row>
@@ -3460,7 +3460,7 @@
     </row>
     <row r="33">
       <c r="C33" s="16" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G33" s="12"/>
     </row>
@@ -3474,7 +3474,7 @@
     </row>
     <row r="35">
       <c r="C35" s="16" t="s">
-        <v>27</v>
+        <v>107</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="12"/>

</xml_diff>